<commit_message>
Updated alignment details -updated inSchool and Partnership target inline with new initial populations -Partnership targets are now loaded from partnered_share_targets.xlsx. -inSchoolAlignment, PartnershipAlignment, FertilityAlignment now use last year Adjustment parameter for a start and also even when alignment process ends (e.g, after 2023 due to lack of target data), the relevant processes (inSchool, Partnership, Fertility) apply this "frozen" adjustment parameter. -adjusted RootSearch exit parameters
</commit_message>
<xml_diff>
--- a/input/inSchool_targets.xlsx
+++ b/input/inSchool_targets.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="6" uniqueCount="2">
   <si>
     <t>year</t>
   </si>
@@ -78,7 +78,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.2934698760509491</v>
+        <v>0.29345935583114624</v>
       </c>
     </row>
     <row r="3">
@@ -86,7 +86,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.30300065875053406</v>
+        <v>0.3029981255531311</v>
       </c>
     </row>
     <row r="4">
@@ -94,7 +94,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.30788367986679077</v>
+        <v>0.30799892544746399</v>
       </c>
     </row>
     <row r="5">
@@ -102,7 +102,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.30556026101112366</v>
+        <v>0.3056219220161438</v>
       </c>
     </row>
     <row r="6">
@@ -110,7 +110,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.29677852988243103</v>
+        <v>0.29676583409309387</v>
       </c>
     </row>
     <row r="7">
@@ -118,7 +118,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.30894365906715393</v>
+        <v>0.30902278423309326</v>
       </c>
     </row>
     <row r="8">
@@ -126,7 +126,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.31126514077186585</v>
+        <v>0.31116059422492981</v>
       </c>
     </row>
     <row r="9">
@@ -134,7 +134,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.30601227283477783</v>
+        <v>0.30586162209510803</v>
       </c>
     </row>
     <row r="10">
@@ -142,7 +142,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.30258682370185852</v>
+        <v>0.3023858368396759</v>
       </c>
     </row>
     <row r="11">
@@ -150,7 +150,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.27610146999359131</v>
+        <v>0.2760101854801178</v>
       </c>
     </row>
     <row r="12">
@@ -158,7 +158,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.27953463792800903</v>
+        <v>0.27926552295684814</v>
       </c>
     </row>
     <row r="13">
@@ -166,7 +166,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.26500150561332703</v>
+        <v>0.26489490270614624</v>
       </c>
     </row>
     <row r="14">
@@ -174,7 +174,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.25127774477005005</v>
+        <v>0.25120154023170471</v>
       </c>
     </row>
   </sheetData>

</xml_diff>